<commit_message>
Agregar asignacion por color de Dry Bag (top 6 colores prioritarios)
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/proyeccion_compra_bags/PROYECCION_COMPRA_6MESES.xlsx
+++ b/proyeccion_compra_bags/PROYECCION_COMPRA_6MESES.xlsx
@@ -10,10 +10,11 @@
     <sheet name="Guia" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Compra_recomendada" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Escenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ventas_mensuales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Estacionalidad" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Colores_mix" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Inventario_detalle" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="DryBag_colores" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Ventas_mensuales" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Estacionalidad" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Colores_mix" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Inventario_detalle" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -977,6 +978,241 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Ventas_hist</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mix_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Inv_actual</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Compra_conservador_3100</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Compra_BASE_3270</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Compra_alto_3470</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>738</v>
+      </c>
+      <c r="C2" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E2" t="n">
+        <v>705</v>
+      </c>
+      <c r="F2" t="n">
+        <v>745</v>
+      </c>
+      <c r="G2" t="n">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>526</v>
+      </c>
+      <c r="C3" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="D3" t="n">
+        <v>21</v>
+      </c>
+      <c r="E3" t="n">
+        <v>495</v>
+      </c>
+      <c r="F3" t="n">
+        <v>524</v>
+      </c>
+      <c r="G3" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>511</v>
+      </c>
+      <c r="C4" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>501</v>
+      </c>
+      <c r="F4" t="n">
+        <v>528</v>
+      </c>
+      <c r="G4" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Azul Rey</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>496</v>
+      </c>
+      <c r="C5" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E5" t="n">
+        <v>465</v>
+      </c>
+      <c r="F5" t="n">
+        <v>492</v>
+      </c>
+      <c r="G5" t="n">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gris Claro</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>464</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" t="n">
+        <v>429</v>
+      </c>
+      <c r="F6" t="n">
+        <v>454</v>
+      </c>
+      <c r="G6" t="n">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Camu</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>423</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>413</v>
+      </c>
+      <c r="F7" t="n">
+        <v>436</v>
+      </c>
+      <c r="G7" t="n">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3158</v>
+      </c>
+      <c r="C8" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" t="n">
+        <v>91</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3008</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3179</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3379</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1253,7 +1489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1997,7 +2233,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2381,7 +2617,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>